<commit_message>
Added the Git setup information
</commit_message>
<xml_diff>
--- a/RoadMap-Requirnments.xlsx
+++ b/RoadMap-Requirnments.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Desktop\Sakshi\Java\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\ClubsKart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{771FA5DE-8CD7-48F9-AF4C-FF8ADEAF9244}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{856DAA86-15C5-4382-A971-F87596183B89}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4FCB8DDC-156F-4E20-A206-55248B33D827}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="GitBash Installation and Setup" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,12 +30,86 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+  <si>
+    <t xml:space="preserve">1. Download Git bash from below link </t>
+  </si>
+  <si>
+    <t>Git for Windows/x64 Setup</t>
+  </si>
+  <si>
+    <t>GitBash Installation and Setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Install with default settings </t>
+  </si>
+  <si>
+    <t xml:space="preserve">only for git commit option choose </t>
+  </si>
+  <si>
+    <t>git commit as-it is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Type GitBash in search bar and open GitBash  </t>
+  </si>
+  <si>
+    <t>4. Type below commands</t>
+  </si>
+  <si>
+    <t>git config --global user.name "Sakshi Galim"</t>
+  </si>
+  <si>
+    <t>git config --global user.email sakshigalim@gmail.com</t>
+  </si>
+  <si>
+    <t>5. check for the details with below command</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> git config --list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. clone the git repo with below command </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">git clone </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://github.com/dipak-c/ClubsKart.git</t>
+    </r>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -58,13 +132,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -78,6 +155,192 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>234960</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>51480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{453DA360-BB2C-4B9C-A8D7-9445CC3B93F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="573548" y="3785419"/>
+          <a:ext cx="9985283" cy="5278964"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>281940</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Rectangle 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F66AA700-1813-46CD-9B4D-147959F288A5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4953000" y="6781800"/>
+          <a:ext cx="2278380" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>209592</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>67426</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>270551</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>158866</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="Speech Bubble: Oval 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE8C3C46-FA17-4D16-9AD3-CF6BEC1F764B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5084753" y="5294910"/>
+          <a:ext cx="1208056" cy="812472"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeEllipseCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -33041"/>
+            <a:gd name="adj2" fmla="val 88720"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>Copy HTTPS</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" baseline="0"/>
+            <a:t> URL</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -377,9 +640,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BBAB418-CC15-4EAE-AD49-954C4EE57A24}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultColWidth="4.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C4" r:id="rId1" display="https://github.com/git-for-windows/git/releases/download/v2.55.0.windows.5/Git-2.55.0.5-64-bit.exe" xr:uid="{4F17E56E-0D1F-4D70-8DC6-C894F04E363A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Modifided Git setup information
</commit_message>
<xml_diff>
--- a/RoadMap-Requirnments.xlsx
+++ b/RoadMap-Requirnments.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\ClubsKart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C846F9BC-9908-4281-AFF9-045D235D1491}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A55723CA-C29E-4F51-800E-B6ED7CB83ED6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4FCB8DDC-156F-4E20-A206-55248B33D827}"/>
   </bookViews>
   <sheets>
-    <sheet name="GitBash Installation and Setup" sheetId="1" r:id="rId1"/>
+    <sheet name="Index" sheetId="2" r:id="rId1"/>
+    <sheet name="GitBash Installation and Setup" sheetId="1" r:id="rId2"/>
+    <sheet name="Roadmap for ClubsKart" sheetId="3" r:id="rId3"/>
+    <sheet name="Requirnment Specification" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,36 +34,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
-  <si>
-    <t xml:space="preserve">1. Download Git bash from below link </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
   <si>
     <t>Git for Windows/x64 Setup</t>
   </si>
   <si>
-    <t>GitBash Installation and Setup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Install with default settings </t>
-  </si>
-  <si>
     <t xml:space="preserve">only for git commit option choose </t>
   </si>
   <si>
-    <t xml:space="preserve">3. Type GitBash in search bar and open GitBash  </t>
-  </si>
-  <si>
-    <t>4. Type below commands</t>
-  </si>
-  <si>
-    <t>5. check for the details with below command</t>
-  </si>
-  <si>
     <t xml:space="preserve"> git config --list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. clone the git repo with below command </t>
   </si>
   <si>
     <r>
@@ -81,9 +63,6 @@
     <t>cd ClubsKart</t>
   </si>
   <si>
-    <t>7. For git commit change to folder clubsKart</t>
-  </si>
-  <si>
     <t>*Add custom msg for commit in ""</t>
   </si>
   <si>
@@ -130,12 +109,6 @@
     </r>
   </si>
   <si>
-    <t>8. SSH Key generation</t>
-  </si>
-  <si>
-    <t>9. Use below command for commiting changes</t>
-  </si>
-  <si>
     <r>
       <t>ssh-keygen -t ed25519 -C "</t>
     </r>
@@ -161,34 +134,7 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">set passpharse - </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>India@123</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">10. For push use below command </t>
-  </si>
-  <si>
     <t>git push</t>
-  </si>
-  <si>
-    <t>9. Add SSH Key to GitHub</t>
-  </si>
-  <si>
-    <t>Key will be generated here on local system</t>
-  </si>
-  <si>
-    <t>c/users</t>
   </si>
   <si>
     <r>
@@ -216,14 +162,287 @@
     </r>
   </si>
   <si>
-    <t>copy this content</t>
+    <t xml:space="preserve">Topics </t>
+  </si>
+  <si>
+    <t>*Replace this name and e-mail 'with yours</t>
+  </si>
+  <si>
+    <t>1. GitBash Installation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1 Download Git bash from below link </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2 Install with default settings </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Type GitBash in search bar and open GitBash  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 Type below commands to set username in git </t>
+  </si>
+  <si>
+    <t>2.3 Check for the git details with below command to confirm setting username is completed</t>
+  </si>
+  <si>
+    <t>3. GitClone</t>
+  </si>
+  <si>
+    <t>2. GitBash Setup</t>
+  </si>
+  <si>
+    <t>3.1 As we will be cloning the Main branch copy HTTPS url</t>
+  </si>
+  <si>
+    <t>3.2 Execute below command on GitBash</t>
+  </si>
+  <si>
+    <t>4. SSH Key generation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.1 Execute below command to create the SSH key </t>
+  </si>
+  <si>
+    <r>
+      <t>4.2 Press Enter when you see message "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Enter file in which to save the key</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <t>c:/users</t>
+  </si>
+  <si>
+    <t>5. Adding the key to Github</t>
+  </si>
+  <si>
+    <t>India@123</t>
+  </si>
+  <si>
+    <t>4.3 Set you passpharse and press enter also enter you passpharse again to confirm</t>
+  </si>
+  <si>
+    <t>4.4 Your key will be generated in below folder</t>
+  </si>
+  <si>
+    <r>
+      <t>5.1 Goto the profile picture section of Github account click "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Settings</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5.2 Goto "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SSH and GPG keys</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">" section </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5.3 Click on "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>New SSH key</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5.4 Copy the contents of "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.pub</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" file saved under "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C:\Users\ACER\.ssh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5.5 In Title set "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Key Dipak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <t>5.6 Paste your copied key in key section</t>
+  </si>
+  <si>
+    <r>
+      <t>5.7 Click on "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Add SSH key</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <t>6. Git Commit</t>
+  </si>
+  <si>
+    <t>6.1 For git commit change to folder ClubsKart on git bash</t>
+  </si>
+  <si>
+    <t>6.2 Use below command for commiting changes to your local repository</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.3 To push changes to web use below command </t>
+  </si>
+  <si>
+    <t>Initial Git setup</t>
+  </si>
+  <si>
+    <t>Requirnment Specification</t>
+  </si>
+  <si>
+    <t>Roadmap for ClubsKart</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -254,6 +473,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -276,11 +504,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -310,7 +542,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>36</xdr:col>
-      <xdr:colOff>234960</xdr:colOff>
+      <xdr:colOff>234961</xdr:colOff>
       <xdr:row>50</xdr:row>
       <xdr:rowOff>51480</xdr:rowOff>
     </xdr:to>
@@ -486,14 +718,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:row>60</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>32</xdr:col>
       <xdr:colOff>208629</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>76456</xdr:rowOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>76455</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -516,7 +748,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="573548" y="10635226"/>
+          <a:off x="548968" y="10635226"/>
           <a:ext cx="8811855" cy="4763165"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -530,14 +762,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>286772</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>49162</xdr:rowOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>32767</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
       <xdr:colOff>163870</xdr:colOff>
-      <xdr:row>67</xdr:row>
-      <xdr:rowOff>90129</xdr:rowOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>73734</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -552,7 +784,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="573546" y="11946194"/>
+          <a:off x="548966" y="12650832"/>
           <a:ext cx="5899356" cy="221225"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -594,16 +826,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>245803</xdr:colOff>
-      <xdr:row>59</xdr:row>
-      <xdr:rowOff>24579</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>237614</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>49162</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>114708</xdr:colOff>
-      <xdr:row>65</xdr:row>
-      <xdr:rowOff>57354</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>188452</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>32774</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -618,13 +850,13 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5981287" y="10659805"/>
-          <a:ext cx="2736647" cy="1114323"/>
+          <a:off x="5374969" y="10864646"/>
+          <a:ext cx="3678902" cy="524386"/>
         </a:xfrm>
         <a:prstGeom prst="wedgeEllipseCallout">
           <a:avLst>
-            <a:gd name="adj1" fmla="val -86933"/>
-            <a:gd name="adj2" fmla="val 63291"/>
+            <a:gd name="adj1" fmla="val -50407"/>
+            <a:gd name="adj2" fmla="val 147666"/>
           </a:avLst>
         </a:prstGeom>
       </xdr:spPr>
@@ -655,7 +887,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-IN" sz="1100" baseline="0"/>
-            <a:t> enter when you see this msg and then enter your passphrase and  enter passphrase again</a:t>
+            <a:t> enter when you see this message</a:t>
           </a:r>
           <a:endParaRPr lang="en-IN" sz="1100"/>
         </a:p>
@@ -667,13 +899,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>88</xdr:row>
+      <xdr:row>123</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>37</xdr:col>
       <xdr:colOff>42903</xdr:colOff>
-      <xdr:row>117</xdr:row>
+      <xdr:row>152</xdr:row>
       <xdr:rowOff>127516</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -711,14 +943,14 @@
     <xdr:from>
       <xdr:col>30</xdr:col>
       <xdr:colOff>122878</xdr:colOff>
-      <xdr:row>105</xdr:row>
-      <xdr:rowOff>98322</xdr:rowOff>
+      <xdr:row>140</xdr:row>
+      <xdr:rowOff>122898</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>36</xdr:col>
       <xdr:colOff>139290</xdr:colOff>
-      <xdr:row>106</xdr:row>
-      <xdr:rowOff>172064</xdr:rowOff>
+      <xdr:row>142</xdr:row>
+      <xdr:rowOff>16382</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -733,7 +965,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8726104" y="19025419"/>
+          <a:off x="8701523" y="25359027"/>
           <a:ext cx="1737057" cy="254000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -777,13 +1009,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>119</xdr:row>
+      <xdr:row>156</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>37</xdr:col>
       <xdr:colOff>42903</xdr:colOff>
-      <xdr:row>148</xdr:row>
+      <xdr:row>185</xdr:row>
       <xdr:rowOff>127516</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -821,13 +1053,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>185148</xdr:colOff>
-      <xdr:row>140</xdr:row>
+      <xdr:row>177</xdr:row>
       <xdr:rowOff>103239</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>201560</xdr:colOff>
-      <xdr:row>141</xdr:row>
+      <xdr:row>178</xdr:row>
       <xdr:rowOff>176981</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -887,13 +1119,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>150</xdr:row>
+      <xdr:row>189</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>37</xdr:col>
       <xdr:colOff>42903</xdr:colOff>
-      <xdr:row>179</xdr:row>
+      <xdr:row>218</xdr:row>
       <xdr:rowOff>127516</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -930,15 +1162,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>30</xdr:col>
-      <xdr:colOff>280193</xdr:colOff>
-      <xdr:row>159</xdr:row>
-      <xdr:rowOff>9832</xdr:rowOff>
+      <xdr:colOff>272000</xdr:colOff>
+      <xdr:row>198</xdr:row>
+      <xdr:rowOff>9831</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>34</xdr:col>
-      <xdr:colOff>90129</xdr:colOff>
-      <xdr:row>160</xdr:row>
-      <xdr:rowOff>122903</xdr:rowOff>
+      <xdr:colOff>81936</xdr:colOff>
+      <xdr:row>199</xdr:row>
+      <xdr:rowOff>122902</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -953,7 +1185,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8883419" y="28670864"/>
+          <a:off x="8850645" y="35700928"/>
           <a:ext cx="957033" cy="293329"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -997,13 +1229,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>181</xdr:row>
+      <xdr:row>255</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>37</xdr:col>
       <xdr:colOff>42903</xdr:colOff>
-      <xdr:row>210</xdr:row>
+      <xdr:row>284</xdr:row>
       <xdr:rowOff>127516</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1027,7 +1259,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="573548" y="32626710"/>
+          <a:off x="548968" y="45965806"/>
           <a:ext cx="10080000" cy="5355000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1040,15 +1272,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>106516</xdr:colOff>
-      <xdr:row>193</xdr:row>
-      <xdr:rowOff>24581</xdr:rowOff>
+      <xdr:colOff>90128</xdr:colOff>
+      <xdr:row>267</xdr:row>
+      <xdr:rowOff>16387</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>203226</xdr:colOff>
-      <xdr:row>194</xdr:row>
-      <xdr:rowOff>137651</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>188450</xdr:colOff>
+      <xdr:row>268</xdr:row>
+      <xdr:rowOff>155677</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1063,74 +1295,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3547806" y="34814387"/>
-          <a:ext cx="957033" cy="293329"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-IN" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>176980</xdr:colOff>
-      <xdr:row>198</xdr:row>
-      <xdr:rowOff>144206</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>200</xdr:row>
-      <xdr:rowOff>77019</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="Rectangle 15">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFADA92D-066A-46DE-BDD8-748A5E550C79}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3618270" y="35835303"/>
-          <a:ext cx="1256891" cy="293329"/>
+          <a:off x="3506838" y="49407097"/>
+          <a:ext cx="2966064" cy="319548"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1171,23 +1337,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>34</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>237618</xdr:colOff>
+      <xdr:row>93</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>64</xdr:col>
-      <xdr:colOff>209575</xdr:colOff>
-      <xdr:row>84</xdr:row>
-      <xdr:rowOff>175349</xdr:rowOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>160418</xdr:colOff>
+      <xdr:row>118</xdr:row>
+      <xdr:rowOff>175348</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Picture 16">
+        <xdr:cNvPr id="22" name="Picture 21">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E627A9DD-0EB0-48D2-8F31-9D79B02DAD36}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87A48B93-6712-488F-801A-AB6989BCF6DE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1203,7 +1369,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9750323" y="10635226"/>
+          <a:off x="499812" y="16764000"/>
           <a:ext cx="8812800" cy="4681800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1215,23 +1381,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>103237</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>127819</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>49167</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>139290</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>49</xdr:col>
-      <xdr:colOff>204839</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>49161</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>150768</xdr:colOff>
+      <xdr:row>100</xdr:row>
+      <xdr:rowOff>60632</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="18" name="Rectangle 17">
+        <xdr:cNvPr id="23" name="Rectangle 22">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9B11673-8910-470C-B5E8-5399EE96C88D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{747BC229-FDAD-42DE-934D-E400C297E198}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1239,7 +1405,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10713882" y="11664335"/>
+          <a:off x="1458457" y="17804580"/>
           <a:ext cx="3542892" cy="281858"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1281,23 +1447,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>39</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>182</xdr:row>
+      <xdr:row>222</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>74</xdr:col>
-      <xdr:colOff>42904</xdr:colOff>
-      <xdr:row>211</xdr:row>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>42903</xdr:colOff>
+      <xdr:row>251</xdr:row>
       <xdr:rowOff>127516</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="Picture 18">
+        <xdr:cNvPr id="24" name="Picture 23">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B1D577E-5676-4CC9-B161-CEB08BC3CA2F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8695436F-EC20-4D37-A549-879A63453AE0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1313,8 +1479,338 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11184194" y="32806968"/>
+          <a:off x="548968" y="40017290"/>
           <a:ext cx="10080000" cy="5355000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>229408</xdr:colOff>
+      <xdr:row>233</xdr:row>
+      <xdr:rowOff>172065</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>40968</xdr:colOff>
+      <xdr:row>236</xdr:row>
+      <xdr:rowOff>90129</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="25" name="Rectangle 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C64C1C50-A926-4F8A-A3D4-87A8E19BBF6A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4219666" y="42172194"/>
+          <a:ext cx="4686721" cy="458838"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>288</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>42903</xdr:colOff>
+      <xdr:row>317</xdr:row>
+      <xdr:rowOff>127517</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="Picture 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{661E2054-070F-4B91-9E55-F5AB712E7382}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="548968" y="51914323"/>
+          <a:ext cx="10080000" cy="5355000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>131097</xdr:colOff>
+      <xdr:row>305</xdr:row>
+      <xdr:rowOff>139290</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>131096</xdr:colOff>
+      <xdr:row>307</xdr:row>
+      <xdr:rowOff>73742</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="28" name="Rectangle 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4DCF087-566D-465C-A550-B6F28E8DCF39}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3547807" y="55118000"/>
+          <a:ext cx="1433870" cy="294968"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>321</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>42903</xdr:colOff>
+      <xdr:row>350</xdr:row>
+      <xdr:rowOff>127516</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Picture 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{03831DDE-98B8-4A79-9F5E-3419F4A08B66}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="548968" y="57862839"/>
+          <a:ext cx="10080000" cy="5355000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>40968</xdr:colOff>
+      <xdr:row>346</xdr:row>
+      <xdr:rowOff>57354</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>155678</xdr:colOff>
+      <xdr:row>348</xdr:row>
+      <xdr:rowOff>16387</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="30" name="Rectangle 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08C62C13-4E67-4209-9F76-0857C89C3908}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3457678" y="62426644"/>
+          <a:ext cx="975032" cy="319549"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>356</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>208629</xdr:colOff>
+      <xdr:row>382</xdr:row>
+      <xdr:rowOff>76455</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Picture 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{476B8F24-3D2D-4539-9FF6-303265505C08}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="548968" y="64171871"/>
+          <a:ext cx="8811855" cy="4763165"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1622,161 +2118,328 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BBAB418-CC15-4EAE-AD49-954C4EE57A24}">
-  <dimension ref="A1:AN217"/>
-  <sheetFormatPr defaultColWidth="4.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{648D0930-0F95-4528-8B30-17F05AE9ECCF}">
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C4" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D8" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="2:35" x14ac:dyDescent="0.3">
-      <c r="B53" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="54" spans="2:35" x14ac:dyDescent="0.3">
-      <c r="C54" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="56" spans="2:35" x14ac:dyDescent="0.3">
-      <c r="B56" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="57" spans="2:35" x14ac:dyDescent="0.3">
-      <c r="C57" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="58" spans="2:35" x14ac:dyDescent="0.3">
-      <c r="C58" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C6" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="AI58" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C10" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="2:35" x14ac:dyDescent="0.3">
-      <c r="AI59" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="60" spans="2:35" x14ac:dyDescent="0.3">
-      <c r="C60" s="3"/>
-    </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B88" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="182" spans="40:40" x14ac:dyDescent="0.3">
-      <c r="AN182" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="205" spans="15:15" x14ac:dyDescent="0.3">
-      <c r="O205" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="213" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B213" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="214" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C214" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="216" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B216" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="217" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C217" t="s">
-        <v>22</v>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C12" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C14" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B16" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B18" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="https://github.com/git-for-windows/git/releases/download/v2.55.0.windows.5/Git-2.55.0.5-64-bit.exe" xr:uid="{4F17E56E-0D1F-4D70-8DC6-C894F04E363A}"/>
+    <hyperlink ref="C4" location="'GitBash Installation and Setup'!A1" display="1. GitBash Installation" xr:uid="{4267CE08-B31F-457D-A5DB-112985D5EEBC}"/>
+    <hyperlink ref="C6" location="'GitBash Installation and Setup'!A9" display="2. GitBash Setup" xr:uid="{010FA8A7-6A3F-41BB-8489-50D31EAE4347}"/>
+    <hyperlink ref="C8" location="'GitBash Installation and Setup'!A19" display="3. GitClone" xr:uid="{530CA766-5BEB-4C99-95F3-2066EF58DCF3}"/>
+    <hyperlink ref="C10" location="'GitBash Installation and Setup'!A55" display="4. SSH Key generation" xr:uid="{F855A38F-E3BD-4B42-9D17-351A78FFB5A0}"/>
+    <hyperlink ref="C12" location="'GitBash Installation and Setup'!A121" display="5. Adding the key to Github" xr:uid="{F221585F-7EDB-42E3-8B77-B02E55DC35EB}"/>
+    <hyperlink ref="C14" location="'GitBash Installation and Setup'!A353" display="6. Git Commit" xr:uid="{0C4B3048-ACEE-4851-AEA4-53F24A0681E9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BBAB418-CC15-4EAE-AD49-954C4EE57A24}">
+  <dimension ref="A1:O389"/>
+  <sheetFormatPr defaultColWidth="4.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>7</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B52" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C53" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B56" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B59" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C61" s="3"/>
+    </row>
+    <row r="88" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B88" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="89" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C89" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="91" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B91" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="92" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C92" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B122" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="155" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B155" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="188" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B188" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="221" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B221" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="254" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B254" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="282" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O282" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="287" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B287" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="320" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B320" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A353" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="354" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B354" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C355" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="385" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B385" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="386" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C386" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="388" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B388" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="389" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C389" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" display="https://github.com/git-for-windows/git/releases/download/v2.55.0.windows.5/Git-2.55.0.5-64-bit.exe" xr:uid="{4F17E56E-0D1F-4D70-8DC6-C894F04E363A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DFF99FF-2F3A-46BC-AB8A-F816B4980A76}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17422BF8-7335-48F5-93BC-E565C95C046C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added Business model sheet
</commit_message>
<xml_diff>
--- a/RoadMap-Requirnments.xlsx
+++ b/RoadMap-Requirnments.xlsx
@@ -1,40 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\ClubsKart\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ClubsKart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59820FD6-5AFA-45B7-8686-2C89FF4A16D2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0464BE73-F1A7-4E59-BDBA-E47E539E1BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2076" yWindow="1716" windowWidth="17280" windowHeight="8880" xr2:uid="{4FCB8DDC-156F-4E20-A206-55248B33D827}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4FCB8DDC-156F-4E20-A206-55248B33D827}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="2" r:id="rId1"/>
     <sheet name="GitBash Installation and Setup" sheetId="1" r:id="rId2"/>
     <sheet name="Roadmap for ClubsKart" sheetId="3" r:id="rId3"/>
     <sheet name="Requirnment Specification" sheetId="4" r:id="rId4"/>
+    <sheet name="Business Model" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
   <si>
     <t>Git for Windows/x64 Setup</t>
   </si>
@@ -434,12 +429,27 @@
   <si>
     <t>Roadmap for ClubsKart</t>
   </si>
+  <si>
+    <t>Git Setup</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Create Flow Chart of complete Business Model</t>
+  </si>
+  <si>
+    <t>Working</t>
+  </si>
+  <si>
+    <t>Business Model</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -479,13 +489,52 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -501,15 +550,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2405,8 +2464,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{648D0930-0F95-4528-8B30-17F05AE9ECCF}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
@@ -2424,35 +2487,32 @@
       <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C5" s="4"/>
-    </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="5" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2464,6 +2524,11 @@
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B20" s="3" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -2608,7 +2673,7 @@
       </c>
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C89" s="5" t="s">
+      <c r="C89" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2712,9 +2777,35 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DFF99FF-2F3A-46BC-AB8A-F816B4980A76}">
-  <dimension ref="A1"/>
+  <dimension ref="B3:G5"/>
   <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="8.21875" style="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="6">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B5" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="6">
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2726,4 +2817,13 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52FFCF2D-4C03-4DC8-AA07-A9142459042D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Hyperlink updated for all sheets, RoadMap and Business Model updated
</commit_message>
<xml_diff>
--- a/RoadMap-Requirnments.xlsx
+++ b/RoadMap-Requirnments.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ClubsKart\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0464BE73-F1A7-4E59-BDBA-E47E539E1BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{423AAEB5-A335-425A-BAC9-CA8D37C42670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4FCB8DDC-156F-4E20-A206-55248B33D827}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Index" sheetId="2" r:id="rId1"/>
     <sheet name="GitBash Installation and Setup" sheetId="1" r:id="rId2"/>
     <sheet name="Roadmap for ClubsKart" sheetId="3" r:id="rId3"/>
-    <sheet name="Requirnment Specification" sheetId="4" r:id="rId4"/>
-    <sheet name="Business Model" sheetId="5" r:id="rId5"/>
+    <sheet name="Business Model" sheetId="4" r:id="rId4"/>
+    <sheet name="Requirnment Specification" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="65">
   <si>
     <t>Git for Windows/x64 Setup</t>
   </si>
@@ -444,12 +444,57 @@
   <si>
     <t>Business Model</t>
   </si>
+  <si>
+    <t>Development of Architecture, Design and Features of App as per Business model</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Backend, API and Database development</t>
+  </si>
+  <si>
+    <t>Front-End Development</t>
+  </si>
+  <si>
+    <t>UI Layout Development</t>
+  </si>
+  <si>
+    <t>UI content and resources gathering (imags, heading, text and other)</t>
+  </si>
+  <si>
+    <t>Selection of Tech-Stack as per 3rd point</t>
+  </si>
+  <si>
+    <t>Implementation in UI</t>
+  </si>
+  <si>
+    <t>Testing and Deployment</t>
+  </si>
+  <si>
+    <t>Testing of all features and functionalities</t>
+  </si>
+  <si>
+    <t>Selection of Deployment Server (Shared hosting, cloud hosting…etc)</t>
+  </si>
+  <si>
+    <t>Deploy on Server</t>
+  </si>
+  <si>
+    <t>Digital Marekting campine setup and execution</t>
+  </si>
+  <si>
+    <t>Go To Sheet</t>
+  </si>
+  <si>
+    <t>Go To Index</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -510,8 +555,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -536,6 +596,36 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -550,13 +640,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -569,6 +657,31 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -597,10 +710,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>36</xdr:col>
-      <xdr:colOff>234961</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>15353</xdr:colOff>
       <xdr:row>50</xdr:row>
-      <xdr:rowOff>51480</xdr:rowOff>
+      <xdr:rowOff>55290</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -778,8 +891,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>208629</xdr:colOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>499213</xdr:colOff>
       <xdr:row>86</xdr:row>
       <xdr:rowOff>76455</xdr:rowOff>
     </xdr:to>
@@ -959,10 +1072,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>42903</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>110069</xdr:colOff>
       <xdr:row>152</xdr:row>
-      <xdr:rowOff>127516</xdr:rowOff>
+      <xdr:rowOff>131326</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1069,10 +1182,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>42903</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>110069</xdr:colOff>
       <xdr:row>185</xdr:row>
-      <xdr:rowOff>127516</xdr:rowOff>
+      <xdr:rowOff>131326</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1179,10 +1292,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>42903</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>110069</xdr:colOff>
       <xdr:row>218</xdr:row>
-      <xdr:rowOff>127516</xdr:rowOff>
+      <xdr:rowOff>131326</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1289,10 +1402,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>42903</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>110069</xdr:colOff>
       <xdr:row>284</xdr:row>
-      <xdr:rowOff>127516</xdr:rowOff>
+      <xdr:rowOff>131326</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1399,10 +1512,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>160418</xdr:colOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>454812</xdr:colOff>
       <xdr:row>118</xdr:row>
-      <xdr:rowOff>175348</xdr:rowOff>
+      <xdr:rowOff>171538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1509,10 +1622,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>42903</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>110069</xdr:colOff>
       <xdr:row>251</xdr:row>
-      <xdr:rowOff>127516</xdr:rowOff>
+      <xdr:rowOff>131326</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1619,10 +1732,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>42903</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>110069</xdr:colOff>
       <xdr:row>317</xdr:row>
-      <xdr:rowOff>127517</xdr:rowOff>
+      <xdr:rowOff>131327</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1729,10 +1842,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>42903</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>110069</xdr:colOff>
       <xdr:row>350</xdr:row>
-      <xdr:rowOff>127516</xdr:rowOff>
+      <xdr:rowOff>131326</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1839,8 +1952,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>208629</xdr:colOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>499213</xdr:colOff>
       <xdr:row>382</xdr:row>
       <xdr:rowOff>76455</xdr:rowOff>
     </xdr:to>
@@ -1883,8 +1996,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>208629</xdr:colOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>499213</xdr:colOff>
       <xdr:row>413</xdr:row>
       <xdr:rowOff>76455</xdr:rowOff>
     </xdr:to>
@@ -1927,8 +2040,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>208629</xdr:colOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>499213</xdr:colOff>
       <xdr:row>444</xdr:row>
       <xdr:rowOff>76455</xdr:rowOff>
     </xdr:to>
@@ -2162,6 +2275,1103 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>247649</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>111702</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Rectangle: Rounded Corners 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F81E220-2999-4349-97E8-E884CF417400}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="508634" y="1266825"/>
+          <a:ext cx="2689168" cy="577215"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Shop Owner</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> Register with our App</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-IN" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>54898</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>54898</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>131445</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Straight Arrow Connector 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35DFC2DD-D624-4C43-B97F-5F12661126F2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="2" idx="2"/>
+          <a:endCxn id="5" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1858933" y="1844040"/>
+          <a:ext cx="0" cy="462915"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>247649</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>135255</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>111702</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="Rectangle: Rounded Corners 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{947E5A45-F23C-42D7-AC06-1A364A58B5F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="508634" y="312420"/>
+          <a:ext cx="2689168" cy="592455"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>START</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>247649</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>135255</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>111702</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Rectangle: Rounded Corners 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{60DB3D95-EF37-47C8-B21F-2F5DB586FF65}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="508634" y="2303145"/>
+          <a:ext cx="2689168" cy="592455"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Shop Owner list All the Producst online</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>135255</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>98022</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Rectangle: Rounded Corners 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{679001B9-E26B-40C3-A3C2-CDDE00D8D97A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4362450" y="312420"/>
+          <a:ext cx="2675487" cy="592455"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Customer</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> filter near by shops as per area pincode</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-IN" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>54898</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>54898</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="7" name="Straight Arrow Connector 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A007C7FD-CD9E-4047-80DF-8D1C82F32B2F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="4" idx="2"/>
+          <a:endCxn id="2" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1858933" y="904875"/>
+          <a:ext cx="0" cy="361950"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>111702</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>65723</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>65723</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="8" name="Connector: Curved 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BBC5959-E387-44B8-AE9F-9A7F4305AF8E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="5" idx="3"/>
+          <a:endCxn id="6" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="3197802" y="606743"/>
+          <a:ext cx="1160838" cy="1990725"/>
+        </a:xfrm>
+        <a:prstGeom prst="curvedConnector3">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:headEnd type="triangle"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>251459</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Rectangle: Rounded Corners 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F1FE792-EBC1-40C2-ACC0-21015B8D8879}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4362449" y="1266825"/>
+          <a:ext cx="2672716" cy="581025"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Customer</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> then s</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>elect Shop and than products list in tha</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>t shop</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-IN" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>44249</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>46672</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="10" name="Straight Arrow Connector 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CCF4F98-BCD5-46AA-A97C-49ABBBB858BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="6" idx="2"/>
+          <a:endCxn id="9" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5704004" y="904875"/>
+          <a:ext cx="2423" cy="361950"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>135255</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>97156</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Rectangle: Rounded Corners 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{112CAC42-FB18-4785-8305-4677C7B46FF3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4371975" y="2303145"/>
+          <a:ext cx="2665096" cy="592455"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Customer Will</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>                                              Add items  &gt;  Payment   &gt;   Checkout</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-IN" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>40005</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>54293</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>135255</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="12" name="Straight Arrow Connector 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{792A242F-FBF1-4B43-A846-5C3F7EEB2D66}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="9" idx="2"/>
+          <a:endCxn id="11" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5697855" y="1847850"/>
+          <a:ext cx="18098" cy="455295"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>211455</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>58017</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19785</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="Rectangle: Rounded Corners 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DC884094-1DCC-45F3-ADF6-0A81E1D27288}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8180070" y="314325"/>
+          <a:ext cx="2675487" cy="787500"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN"/>
+            <a:t>Orders placed </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" b="1"/>
+            <a:t>before 11:00 AM</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN"/>
+            <a:t> will be delivered at </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" b="1"/>
+            <a:t>1:00 PM</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN"/>
+            <a:t>, while orders placed </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" b="1"/>
+            <a:t>from 11:00 AM to midnight</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN"/>
+            <a:t> will be delivered by </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" b="1"/>
+            <a:t>9:00 AM the next morning</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN"/>
+            <a:t>.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>93346</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>165150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>211455</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>65723</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="14" name="Connector: Curved 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7063CF57-9588-4710-BA3D-427DC0E0FA0B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="11" idx="3"/>
+          <a:endCxn id="13" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="7040881" y="711885"/>
+          <a:ext cx="1139189" cy="1885583"/>
+        </a:xfrm>
+        <a:prstGeom prst="curvedConnector3">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:headEnd type="triangle"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>211454</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>177165</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>53340</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="Rectangle: Rounded Corners 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BE48A66-939F-440C-8ED5-E66CD5678CA0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8180069" y="1259205"/>
+          <a:ext cx="2678431" cy="784860"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>END</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>3810</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19785</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>6149</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>177165</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="16" name="Straight Arrow Connector 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E01BA00-B3A9-4EC1-9EAC-219A8C7295B3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+          <a:stCxn id="13" idx="2"/>
+          <a:endCxn id="15" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="9521190" y="1101825"/>
+          <a:ext cx="2339" cy="157380"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2464,74 +3674,186 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{648D0930-0F95-4528-8B30-17F05AE9ECCF}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
         <v>11</v>
       </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="17"/>
+      <c r="B2" s="17" t="s">
         <v>42</v>
       </c>
+      <c r="C2" s="16"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C4" s="4" t="s">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="15" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+    </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C6" s="5" t="s">
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="15" t="s">
         <v>20</v>
       </c>
     </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+    </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C8" s="5" t="s">
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="15" t="s">
         <v>19</v>
       </c>
     </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+    </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C10" s="5" t="s">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="15" t="s">
         <v>23</v>
       </c>
     </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+    </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C12" s="5" t="s">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="15" t="s">
         <v>27</v>
       </c>
     </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+    </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C14" s="5" t="s">
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B16" s="3" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+    </row>
+    <row r="16" spans="1:3" s="12" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="16"/>
+      <c r="B17" s="17" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B18" s="3" t="s">
+      <c r="C17" s="16"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="14"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="14"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+    </row>
+    <row r="21" spans="1:3" s="12" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="16"/>
+      <c r="B22" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="16"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="14"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="14"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="14"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="14"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="18"/>
+    </row>
+    <row r="26" spans="1:3" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="20"/>
+      <c r="C26" s="21"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="16"/>
+      <c r="B27" s="17" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B20" s="3" t="s">
-        <v>49</v>
-      </c>
+      <c r="C27" s="16"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="14"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="14"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="C4" location="'GitBash Installation and Setup'!A1" display="1. GitBash Installation" xr:uid="{4267CE08-B31F-457D-A5DB-112985D5EEBC}"/>
     <hyperlink ref="C6" location="'GitBash Installation and Setup'!A9" display="2. GitBash Setup" xr:uid="{010FA8A7-6A3F-41BB-8489-50D31EAE4347}"/>
@@ -2539,6 +3861,9 @@
     <hyperlink ref="C10" location="'GitBash Installation and Setup'!A55" display="4. SSH Key generation" xr:uid="{F855A38F-E3BD-4B42-9D17-351A78FFB5A0}"/>
     <hyperlink ref="C12" location="'GitBash Installation and Setup'!A121" display="5. Adding the key to Github" xr:uid="{F221585F-7EDB-42E3-8B77-B02E55DC35EB}"/>
     <hyperlink ref="C14" location="'GitBash Installation and Setup'!A353" display="6. Git Commit" xr:uid="{0C4B3048-ACEE-4851-AEA4-53F24A0681E9}"/>
+    <hyperlink ref="C19" location="'Roadmap for ClubsKart'!A1" display="Go To Sheet" xr:uid="{E3E4FA66-3DEF-4A1C-AF9A-1F2FE1A07B25}"/>
+    <hyperlink ref="C29" location="'Requirnment Specification'!A1" display="Go To Sheet" xr:uid="{1A6F0198-0546-49D4-8C35-D8F8A6742FBB}"/>
+    <hyperlink ref="C24" location="'Business Model'!A1" display="Go To Sheet" xr:uid="{9FBB058A-6686-4CB6-91D3-9E37EBBF961C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2546,62 +3871,68 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BBAB418-CC15-4EAE-AD49-954C4EE57A24}">
-  <dimension ref="A1:O417"/>
+  <dimension ref="A1:AH417"/>
   <sheetFormatPr defaultColWidth="4.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" customWidth="1"/>
+    <col min="32" max="32" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="AF1" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="AG1" s="12"/>
+      <c r="AH1" s="12"/>
+    </row>
+    <row r="2" spans="1:34" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.3">
       <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.3">
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:34" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:34" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:34" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>6</v>
       </c>
@@ -2609,12 +3940,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:34" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:34" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>18</v>
       </c>
@@ -2768,6 +4099,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="https://github.com/git-for-windows/git/releases/download/v2.55.0.windows.5/Git-2.55.0.5-64-bit.exe" xr:uid="{4F17E56E-0D1F-4D70-8DC6-C894F04E363A}"/>
+    <hyperlink ref="AF1" location="Index!A1" display="Go To Index" xr:uid="{BF6B5060-8FC1-4B0A-962B-50308D635E46}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -2777,53 +4109,232 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DFF99FF-2F3A-46BC-AB8A-F816B4980A76}">
-  <dimension ref="B3:G5"/>
+  <dimension ref="B1:AH29"/>
   <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="8.21875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B3" s="7" t="s">
+    <row r="1" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="AF1" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="AG1" s="12"/>
+      <c r="AH1" s="12"/>
+    </row>
+    <row r="3" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="B3" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="4">
         <v>1</v>
       </c>
       <c r="G3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B5" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="6">
+    <row r="5" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="4">
         <v>2</v>
       </c>
       <c r="G5" t="s">
         <v>47</v>
       </c>
     </row>
+    <row r="7" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="B7" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="4">
+        <v>3</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="B9" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" s="4">
+        <v>4</v>
+      </c>
+      <c r="G9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="AH10" s="3"/>
+    </row>
+    <row r="11" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="B11" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="4">
+        <v>5</v>
+      </c>
+      <c r="G11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="B13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="4">
+        <v>6</v>
+      </c>
+      <c r="G13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="2:34" x14ac:dyDescent="0.3">
+      <c r="B15" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G15" s="9">
+        <v>6.1</v>
+      </c>
+      <c r="I15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G17" s="9">
+        <v>6.2</v>
+      </c>
+      <c r="I17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B19" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" s="9">
+        <v>6.3</v>
+      </c>
+      <c r="I19" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="11"/>
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B21" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E21" s="4">
+        <v>7</v>
+      </c>
+      <c r="G21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G23" s="9">
+        <v>7.1</v>
+      </c>
+      <c r="I23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B25" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G25" s="9">
+        <v>7.2</v>
+      </c>
+      <c r="I25" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G27" s="9">
+        <v>7.3</v>
+      </c>
+      <c r="I27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B29" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E29" s="4">
+        <v>8</v>
+      </c>
+      <c r="G29" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="AF1" location="Index!A1" display="Go To Index" xr:uid="{63AAAA3F-B2B0-4943-BB04-6AEFE33E8824}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17422BF8-7335-48F5-93BC-E565C95C046C}">
-  <dimension ref="A1"/>
+  <dimension ref="AU1:AW1"/>
   <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="47" max="47" width="11.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="47:49" x14ac:dyDescent="0.3">
+      <c r="AU1" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="AV1" s="12"/>
+      <c r="AW1" s="12"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="AU1" location="Index!A1" display="Go To Index" xr:uid="{00BD06DA-DF10-4D31-B718-04F4A6AE5830}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52FFCF2D-4C03-4DC8-AA07-A9142459042D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6057F326-C659-485E-9A34-1896A8E6494E}">
+  <dimension ref="AF1:AH1"/>
+  <sheetFormatPr defaultColWidth="3.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="32" max="32" width="11.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="32:34" x14ac:dyDescent="0.3">
+      <c r="AF1" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="AG1" s="12"/>
+      <c r="AH1" s="12"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="AF1" location="Index!A1" display="Go To Index" xr:uid="{5501FA03-2A64-4026-963C-98A4735D85F9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>